<commit_message>
fix: mark stale demos offline
</commit_message>
<xml_diff>
--- a/bir_portfolio.xlsx
+++ b/bir_portfolio.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="Rd902371427b14869"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" r:id="R90ee66bcf3294c29"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verified Working" sheetId="3" r:id="R9ca7ce6e5e7141a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing Limitations" sheetId="4" r:id="R0e3256265e3a48ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" r:id="R40d96dc312d4428a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="2" r:id="R0dd688441be7413d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verified Working" sheetId="3" r:id="R08975fc02cbd4960"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testing Limitations" sheetId="4" r:id="R0d9295e2ea394a5a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -681,6 +681,18 @@
           <x:t xml:space="preserve">No code fix needed. Manually hit the live demo once to confirm it wakes up; if it stays unresponsive, treat like the prior hard-down incident (badge back to 'Demo offline').</x:t>
         </x:is>
       </x:c>
+      <x:c r="H3" s="13" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="I3" s="12" t="str">
+        <x:v>Root cause: status.json had stale CraveConnect=true while the endpoint timed out; the UI also trusted stale true values. Fix: updated status.json to observed offline state and added stale-health handling so old online checks render as Status stale instead of online.</x:v>
+      </x:c>
+      <x:c r="J3" s="12" t="str">
+        <x:v>Verified direct curl probes: SemantiCache API and CraveConnect both timed out at 150s. Local page with v=18 showed iORA DocQA, SemantiCache, and CraveConnect as offline; no horizontal overflow; node --check and git diff --check passed.</x:v>
+      </x:c>
+      <x:c r="K3" s="12" t="str">
+        <x:v>2026-07-25 01:30</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>